<commit_message>
Implemented and confirmed writing all memory field types from the Program Memory tab
</commit_message>
<xml_diff>
--- a/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
+++ b/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\matt\Code\gtr2-memory-operations-tool-wpf\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D96718A6-AA9E-4843-BE04-363A764D29CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAFF128-FD19-428D-9448-10D9F3F2749E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10812" yWindow="5424" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
+    <workbookView xWindow="19188" yWindow="8616" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Gtr2MemVehSlot-fields-python-r4" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="290">
   <si>
     <t>Name</t>
   </si>
@@ -957,6 +957,15 @@
   </si>
   <si>
     <t>sim_gdb_Category_Tag_Name</t>
+  </si>
+  <si>
+    <t>Confirmed (260414): Last Laptime</t>
+  </si>
+  <si>
+    <t>Confirmed (260414): Session Best Laptime. Displayed in Grid tab. Displayed in Timing tab but breaks display when changed.</t>
+  </si>
+  <si>
+    <t>Timing &gt; Sectors screen has Split Time which might be around this area</t>
   </si>
 </sst>
 </file>
@@ -1453,7 +1462,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="8" xfId="15" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1461,6 +1470,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="17"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="18"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" xfId="13"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5740,7 +5750,7 @@
       </c>
       <c r="I157" s="1"/>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="4" t="s">
         <v>164</v>
       </c>
@@ -5766,8 +5776,8 @@
       </c>
       <c r="I158" s="1"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A159" s="4" t="s">
+    <row r="159" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A159" s="5" t="s">
         <v>165</v>
       </c>
       <c r="B159" t="s">
@@ -5787,9 +5797,11 @@
         <f t="shared" si="5"/>
         <v>19304</v>
       </c>
-      <c r="I159" s="1"/>
-    </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I159" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A160" s="4" t="s">
         <v>166</v>
       </c>
@@ -6071,7 +6083,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="4" t="s">
         <v>177</v>
       </c>
@@ -6099,8 +6111,8 @@
         <v>278</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A172" s="4" t="s">
+    <row r="172" spans="1:9" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A172" s="5" t="s">
         <v>178</v>
       </c>
       <c r="B172" t="s">
@@ -6120,9 +6132,11 @@
         <f t="shared" si="5"/>
         <v>19436</v>
       </c>
-      <c r="I172" s="1"/>
-    </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I172" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
         <v>179</v>
       </c>
@@ -6214,7 +6228,7 @@
       </c>
       <c r="I176" s="1"/>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="4" t="s">
         <v>183</v>
       </c>
@@ -6237,8 +6251,8 @@
       </c>
       <c r="I177" s="1"/>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A178" s="4" t="s">
+    <row r="178" spans="1:9" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A178" s="5" t="s">
         <v>184</v>
       </c>
       <c r="B178" t="s">
@@ -6261,9 +6275,11 @@
       <c r="G178">
         <v>19460</v>
       </c>
-      <c r="I178" s="1"/>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I178" s="1" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A179" s="4" t="s">
         <v>185</v>
       </c>

</xml_diff>

<commit_message>
Figure out much faster GTR2 Grid Slots memory reading for Automatic AI tab
</commit_message>
<xml_diff>
--- a/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
+++ b/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\matt\Code\gtr2-memory-operations-tool-wpf\etc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAFF128-FD19-428D-9448-10D9F3F2749E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F36E81E-EE5B-430B-AC6D-3105EE398689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19188" yWindow="8616" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
+    <workbookView xWindow="17532" yWindow="3972" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Gtr2MemVehSlot-fields-python-r4" sheetId="1" r:id="rId1"/>
@@ -1857,15 +1857,15 @@
   <dimension ref="A1:I270"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="54.109375" customWidth="1"/>
+    <col min="9" max="9" width="53.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Automatic AI tab now reads driver class with minimal memory fields to make it fast (100ms). Now able to read and display drivers and their last lap time in a DataGrid.
</commit_message>
<xml_diff>
--- a/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
+++ b/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\matt\Code\gtr2-memory-operations-tool-wpf\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F36E81E-EE5B-430B-AC6D-3105EE398689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FBD10A-08EF-4557-826C-F7D4B68CA63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17532" yWindow="3972" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="295">
   <si>
     <t>Name</t>
   </si>
@@ -941,9 +941,6 @@
     <t>Verified in Gtr2MemOpsTool gui app.</t>
   </si>
   <si>
-    <t>FIXME: Field Length = 40 not 36 (confirmed reading driver names correctly in Gtr2MemOpsTool gui app)</t>
-  </si>
-  <si>
     <t>Verified in Gtr2MemOpsTool gui app;</t>
   </si>
   <si>
@@ -959,13 +956,31 @@
     <t>sim_gdb_Category_Tag_Name</t>
   </si>
   <si>
-    <t>Confirmed (260414): Last Laptime</t>
-  </si>
-  <si>
     <t>Confirmed (260414): Session Best Laptime. Displayed in Grid tab. Displayed in Timing tab but breaks display when changed.</t>
   </si>
   <si>
     <t>Timing &gt; Sectors screen has Split Time which might be around this area</t>
+  </si>
+  <si>
+    <t>Quirks:</t>
+  </si>
+  <si>
+    <t>- Laptimes can be -1 (no lap time)'</t>
+  </si>
+  <si>
+    <t>Gotchas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed (260414): Last Laptime; </t>
+  </si>
+  <si>
+    <t>-1:No lap time?</t>
+  </si>
+  <si>
+    <t>-1: No lap time (Confirmed)</t>
+  </si>
+  <si>
+    <t>Note: Field Length = 40 not 36 (confirmed reading driver names correctly in Gtr2MemOpsTool gui app)</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1136,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1301,6 +1316,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1418,7 +1439,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1461,8 +1482,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="33" borderId="0" applyFont="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="8" xfId="15" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1471,8 +1493,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="18"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="7" xfId="13"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1499,6 +1522,7 @@
     <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Caution" xfId="42" xr:uid="{FAA8E316-8CC9-4C9F-8303-79C01072CD48}"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
@@ -1854,10 +1878,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C11D8C-D518-42C3-A7D3-6BD4B138053A}">
-  <dimension ref="A1:I270"/>
+  <dimension ref="A1:J272"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
@@ -1866,9 +1890,10 @@
     <col min="7" max="7" width="18.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1896,8 +1921,11 @@
       <c r="I1" s="4" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J1" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1918,8 +1946,9 @@
         <v>0</v>
       </c>
       <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -1941,8 +1970,9 @@
         <v>4</v>
       </c>
       <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -1964,8 +1994,9 @@
         <v>8</v>
       </c>
       <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -1987,8 +2018,9 @@
         <v>12</v>
       </c>
       <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
@@ -2010,8 +2042,9 @@
         <v>16</v>
       </c>
       <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -2033,8 +2066,9 @@
         <v>20</v>
       </c>
       <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
@@ -2056,8 +2090,9 @@
         <v>24</v>
       </c>
       <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -2079,8 +2114,9 @@
         <v>28</v>
       </c>
       <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
@@ -2102,8 +2138,9 @@
         <v>32</v>
       </c>
       <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
@@ -2131,8 +2168,9 @@
         <v>184</v>
       </c>
       <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>19</v>
       </c>
@@ -2154,8 +2192,9 @@
         <v>184</v>
       </c>
       <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
@@ -2183,8 +2222,9 @@
         <v>2792</v>
       </c>
       <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>21</v>
       </c>
@@ -2206,8 +2246,9 @@
         <v>2792</v>
       </c>
       <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>22</v>
       </c>
@@ -2235,8 +2276,9 @@
         <v>5256</v>
       </c>
       <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
@@ -2258,8 +2300,9 @@
         <v>5256</v>
       </c>
       <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>24</v>
       </c>
@@ -2281,8 +2324,9 @@
         <v>5260</v>
       </c>
       <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
@@ -2304,8 +2348,9 @@
         <v>5516</v>
       </c>
       <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>26</v>
       </c>
@@ -2327,8 +2372,9 @@
         <v>5520</v>
       </c>
       <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>27</v>
       </c>
@@ -2350,8 +2396,9 @@
         <v>5524</v>
       </c>
       <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>28</v>
       </c>
@@ -2373,8 +2420,9 @@
         <v>5536</v>
       </c>
       <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>29</v>
       </c>
@@ -2402,8 +2450,9 @@
         <v>5572</v>
       </c>
       <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>30</v>
       </c>
@@ -2425,8 +2474,9 @@
         <v>5572</v>
       </c>
       <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
@@ -2454,8 +2504,9 @@
         <v>5596</v>
       </c>
       <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>32</v>
       </c>
@@ -2477,8 +2528,9 @@
         <v>5596</v>
       </c>
       <c r="I25" s="1"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>33</v>
       </c>
@@ -2506,8 +2558,9 @@
         <v>5620</v>
       </c>
       <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>34</v>
       </c>
@@ -2535,8 +2588,9 @@
         <v>5688</v>
       </c>
       <c r="I27" s="1"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>35</v>
       </c>
@@ -2558,8 +2612,9 @@
         <v>5688</v>
       </c>
       <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>36</v>
       </c>
@@ -2584,8 +2639,9 @@
         <v>5692</v>
       </c>
       <c r="I29" s="1"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J29" s="1"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>37</v>
       </c>
@@ -2610,8 +2666,9 @@
         <v>5696</v>
       </c>
       <c r="I30" s="1"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J30" s="1"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>38</v>
       </c>
@@ -2636,8 +2693,9 @@
         <v>5700</v>
       </c>
       <c r="I31" s="1"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J31" s="1"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>39</v>
       </c>
@@ -2665,8 +2723,9 @@
         <v>5708</v>
       </c>
       <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J32" s="1"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>40</v>
       </c>
@@ -2688,8 +2747,9 @@
         <v>5708</v>
       </c>
       <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J33" s="1"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>41</v>
       </c>
@@ -2711,8 +2771,9 @@
         <v>5720</v>
       </c>
       <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J34" s="1"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>42</v>
       </c>
@@ -2734,8 +2795,9 @@
         <v>5732</v>
       </c>
       <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J35" s="1"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>43</v>
       </c>
@@ -2763,8 +2825,9 @@
         <v>5760</v>
       </c>
       <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J36" s="1"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>44</v>
       </c>
@@ -2786,8 +2849,9 @@
         <v>5760</v>
       </c>
       <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J37" s="1"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>45</v>
       </c>
@@ -2809,8 +2873,9 @@
         <v>5761</v>
       </c>
       <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J38" s="1"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>46</v>
       </c>
@@ -2832,8 +2897,9 @@
         <v>5762</v>
       </c>
       <c r="I39" s="1"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J39" s="1"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>47</v>
       </c>
@@ -2855,8 +2921,9 @@
         <v>5763</v>
       </c>
       <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J40" s="1"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>48</v>
       </c>
@@ -2878,8 +2945,9 @@
         <v>5764</v>
       </c>
       <c r="I41" s="1"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J41" s="1"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>49</v>
       </c>
@@ -2901,8 +2969,9 @@
         <v>5765</v>
       </c>
       <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J42" s="1"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>50</v>
       </c>
@@ -2924,8 +2993,9 @@
         <v>5766</v>
       </c>
       <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J43" s="1"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>51</v>
       </c>
@@ -2947,8 +3017,9 @@
         <v>5767</v>
       </c>
       <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J44" s="1"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>52</v>
       </c>
@@ -2976,8 +3047,9 @@
         <v>5776</v>
       </c>
       <c r="I45" s="1"/>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J45" s="1"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>53</v>
       </c>
@@ -2999,8 +3071,9 @@
         <v>5776</v>
       </c>
       <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J46" s="1"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>54</v>
       </c>
@@ -3028,8 +3101,9 @@
         <v>5804</v>
       </c>
       <c r="I47" s="1"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J47" s="1"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>55</v>
       </c>
@@ -3051,8 +3125,9 @@
         <v>5804</v>
       </c>
       <c r="I48" s="1"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J48" s="1"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>56</v>
       </c>
@@ -3077,8 +3152,9 @@
         <v>5816</v>
       </c>
       <c r="I49" s="1"/>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J49" s="1"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>57</v>
       </c>
@@ -3100,8 +3176,9 @@
         <v>5832</v>
       </c>
       <c r="I50" s="1"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J50" s="1"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>58</v>
       </c>
@@ -3126,8 +3203,9 @@
         <v>5844</v>
       </c>
       <c r="I51" s="1"/>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J51" s="1"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>59</v>
       </c>
@@ -3149,8 +3227,9 @@
         <v>5860</v>
       </c>
       <c r="I52" s="1"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J52" s="1"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>60</v>
       </c>
@@ -3175,8 +3254,9 @@
         <v>5872</v>
       </c>
       <c r="I53" s="1"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J53" s="1"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>61</v>
       </c>
@@ -3198,8 +3278,9 @@
         <v>5888</v>
       </c>
       <c r="I54" s="1"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J54" s="1"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>62</v>
       </c>
@@ -3224,8 +3305,9 @@
         <v>5900</v>
       </c>
       <c r="I55" s="1"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J55" s="1"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>63</v>
       </c>
@@ -3247,8 +3329,9 @@
         <v>5916</v>
       </c>
       <c r="I56" s="1"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J56" s="1"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>64</v>
       </c>
@@ -3273,8 +3356,9 @@
         <v>5928</v>
       </c>
       <c r="I57" s="1"/>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J57" s="1"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>65</v>
       </c>
@@ -3296,8 +3380,9 @@
         <v>5944</v>
       </c>
       <c r="I58" s="1"/>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J58" s="1"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>66</v>
       </c>
@@ -3322,8 +3407,9 @@
         <v>5956</v>
       </c>
       <c r="I59" s="1"/>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J59" s="1"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>67</v>
       </c>
@@ -3345,8 +3431,9 @@
         <v>5972</v>
       </c>
       <c r="I60" s="1"/>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J60" s="1"/>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>62</v>
       </c>
@@ -3371,8 +3458,9 @@
         <v>5984</v>
       </c>
       <c r="I61" s="1"/>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J61" s="1"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>68</v>
       </c>
@@ -3394,8 +3482,9 @@
         <v>6000</v>
       </c>
       <c r="I62" s="1"/>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J62" s="1"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>69</v>
       </c>
@@ -3420,8 +3509,9 @@
         <v>6012</v>
       </c>
       <c r="I63" s="1"/>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J63" s="1"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>70</v>
       </c>
@@ -3443,8 +3533,9 @@
         <v>6028</v>
       </c>
       <c r="I64" s="1"/>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J64" s="1"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>71</v>
       </c>
@@ -3469,8 +3560,9 @@
         <v>6040</v>
       </c>
       <c r="I65" s="1"/>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J65" s="1"/>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>72</v>
       </c>
@@ -3492,8 +3584,9 @@
         <v>6056</v>
       </c>
       <c r="I66" s="1"/>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J66" s="1"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>73</v>
       </c>
@@ -3518,8 +3611,9 @@
         <v>6068</v>
       </c>
       <c r="I67" s="1"/>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J67" s="1"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>74</v>
       </c>
@@ -3541,8 +3635,9 @@
         <v>6084</v>
       </c>
       <c r="I68" s="1"/>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J68" s="1"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>75</v>
       </c>
@@ -3567,8 +3662,9 @@
         <v>6096</v>
       </c>
       <c r="I69" s="1"/>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J69" s="1"/>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>76</v>
       </c>
@@ -3590,8 +3686,9 @@
         <v>6112</v>
       </c>
       <c r="I70" s="1"/>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J70" s="1"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>77</v>
       </c>
@@ -3616,8 +3713,9 @@
         <v>6124</v>
       </c>
       <c r="I71" s="1"/>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J71" s="1"/>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>78</v>
       </c>
@@ -3639,8 +3737,9 @@
         <v>6140</v>
       </c>
       <c r="I72" s="1"/>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J72" s="1"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>79</v>
       </c>
@@ -3665,8 +3764,9 @@
         <v>6152</v>
       </c>
       <c r="I73" s="1"/>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J73" s="1"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>80</v>
       </c>
@@ -3688,8 +3788,9 @@
         <v>6168</v>
       </c>
       <c r="I74" s="1"/>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J74" s="1"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>81</v>
       </c>
@@ -3714,8 +3815,9 @@
         <v>6180</v>
       </c>
       <c r="I75" s="1"/>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J75" s="1"/>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>82</v>
       </c>
@@ -3737,8 +3839,9 @@
         <v>6196</v>
       </c>
       <c r="I76" s="1"/>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J76" s="1"/>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>83</v>
       </c>
@@ -3763,8 +3866,9 @@
         <v>6208</v>
       </c>
       <c r="I77" s="1"/>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J77" s="1"/>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>84</v>
       </c>
@@ -3786,8 +3890,9 @@
         <v>6224</v>
       </c>
       <c r="I78" s="1"/>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J78" s="1"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>85</v>
       </c>
@@ -3812,8 +3917,9 @@
         <v>6236</v>
       </c>
       <c r="I79" s="1"/>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J79" s="1"/>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>86</v>
       </c>
@@ -3835,8 +3941,9 @@
         <v>6252</v>
       </c>
       <c r="I80" s="1"/>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J80" s="1"/>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>87</v>
       </c>
@@ -3861,8 +3968,9 @@
         <v>6264</v>
       </c>
       <c r="I81" s="1"/>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J81" s="1"/>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>88</v>
       </c>
@@ -3884,8 +3992,9 @@
         <v>6280</v>
       </c>
       <c r="I82" s="1"/>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J82" s="1"/>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>89</v>
       </c>
@@ -3910,8 +4019,9 @@
         <v>6292</v>
       </c>
       <c r="I83" s="1"/>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J83" s="1"/>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>90</v>
       </c>
@@ -3933,8 +4043,9 @@
         <v>6308</v>
       </c>
       <c r="I84" s="1"/>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J84" s="1"/>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>91</v>
       </c>
@@ -3959,8 +4070,9 @@
         <v>6320</v>
       </c>
       <c r="I85" s="1"/>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J85" s="1"/>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>92</v>
       </c>
@@ -3982,8 +4094,9 @@
         <v>6336</v>
       </c>
       <c r="I86" s="1"/>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J86" s="1"/>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>93</v>
       </c>
@@ -4008,8 +4121,9 @@
         <v>6348</v>
       </c>
       <c r="I87" s="1"/>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J87" s="1"/>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>94</v>
       </c>
@@ -4031,8 +4145,9 @@
         <v>6364</v>
       </c>
       <c r="I88" s="1"/>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J88" s="1"/>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>95</v>
       </c>
@@ -4057,8 +4172,9 @@
         <v>6376</v>
       </c>
       <c r="I89" s="1"/>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J89" s="1"/>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>96</v>
       </c>
@@ -4080,8 +4196,9 @@
         <v>6392</v>
       </c>
       <c r="I90" s="1"/>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J90" s="1"/>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>97</v>
       </c>
@@ -4106,8 +4223,9 @@
         <v>6404</v>
       </c>
       <c r="I91" s="1"/>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J91" s="1"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>98</v>
       </c>
@@ -4129,8 +4247,9 @@
         <v>6420</v>
       </c>
       <c r="I92" s="1"/>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J92" s="1"/>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>99</v>
       </c>
@@ -4155,8 +4274,9 @@
         <v>6432</v>
       </c>
       <c r="I93" s="1"/>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J93" s="1"/>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>100</v>
       </c>
@@ -4178,8 +4298,9 @@
         <v>6448</v>
       </c>
       <c r="I94" s="1"/>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J94" s="1"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>101</v>
       </c>
@@ -4204,8 +4325,9 @@
         <v>6460</v>
       </c>
       <c r="I95" s="1"/>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J95" s="1"/>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>102</v>
       </c>
@@ -4227,8 +4349,9 @@
         <v>6476</v>
       </c>
       <c r="I96" s="1"/>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J96" s="1"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>103</v>
       </c>
@@ -4253,8 +4376,9 @@
         <v>6488</v>
       </c>
       <c r="I97" s="1"/>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J97" s="1"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>104</v>
       </c>
@@ -4282,8 +4406,9 @@
         <v>6572</v>
       </c>
       <c r="I98" s="1"/>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J98" s="1"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>105</v>
       </c>
@@ -4305,8 +4430,9 @@
         <v>6572</v>
       </c>
       <c r="I99" s="1"/>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J99" s="1"/>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>106</v>
       </c>
@@ -4328,8 +4454,9 @@
         <v>6576</v>
       </c>
       <c r="I100" s="1"/>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J100" s="1"/>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>107</v>
       </c>
@@ -4357,8 +4484,9 @@
         <v>14808</v>
       </c>
       <c r="I101" s="1"/>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J101" s="1"/>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>108</v>
       </c>
@@ -4386,8 +4514,9 @@
         <v>15616</v>
       </c>
       <c r="I102" s="1"/>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J102" s="1"/>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>109</v>
       </c>
@@ -4409,8 +4538,9 @@
         <v>15616</v>
       </c>
       <c r="I103" s="1"/>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J103" s="1"/>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>110</v>
       </c>
@@ -4438,8 +4568,9 @@
         <v>15884</v>
       </c>
       <c r="I104" s="1"/>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J104" s="1"/>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>111</v>
       </c>
@@ -4461,8 +4592,9 @@
         <v>15884</v>
       </c>
       <c r="I105" s="1"/>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J105" s="1"/>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
         <v>112</v>
       </c>
@@ -4490,8 +4622,9 @@
         <v>15928</v>
       </c>
       <c r="I106" s="1"/>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J106" s="1"/>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
         <v>113</v>
       </c>
@@ -4515,8 +4648,9 @@
       <c r="I107" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J107" s="1"/>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>114</v>
       </c>
@@ -4544,8 +4678,9 @@
         <v>15988</v>
       </c>
       <c r="I108" s="1"/>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J108" s="1"/>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>115</v>
       </c>
@@ -4567,8 +4702,9 @@
         <v>15988</v>
       </c>
       <c r="I109" s="1"/>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J109" s="1"/>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>116</v>
       </c>
@@ -4596,8 +4732,9 @@
         <v>16048</v>
       </c>
       <c r="I110" s="1"/>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J110" s="1"/>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>117</v>
       </c>
@@ -4621,8 +4758,9 @@
       <c r="I111" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J111" s="1"/>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>118</v>
       </c>
@@ -4647,8 +4785,9 @@
         <v>16052</v>
       </c>
       <c r="I112" s="1"/>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J112" s="1"/>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>119</v>
       </c>
@@ -4673,8 +4812,9 @@
         <v>16056</v>
       </c>
       <c r="I113" s="1"/>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J113" s="1"/>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
         <v>120</v>
       </c>
@@ -4696,8 +4836,9 @@
         <v>16060</v>
       </c>
       <c r="I114" s="1"/>
-    </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J114" s="1"/>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>121</v>
       </c>
@@ -4722,8 +4863,9 @@
         <v>16072</v>
       </c>
       <c r="I115" s="1"/>
-    </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J115" s="1"/>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>122</v>
       </c>
@@ -4745,8 +4887,9 @@
         <v>16076</v>
       </c>
       <c r="I116" s="1"/>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J116" s="1"/>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>123</v>
       </c>
@@ -4771,8 +4914,9 @@
         <v>16080</v>
       </c>
       <c r="I117" s="1"/>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J117" s="1"/>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>124</v>
       </c>
@@ -4796,8 +4940,9 @@
       <c r="I118" s="1" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J118" s="1"/>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>125</v>
       </c>
@@ -4825,8 +4970,9 @@
         <v>16136</v>
       </c>
       <c r="I119" s="1"/>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J119" s="1"/>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>126</v>
       </c>
@@ -4850,8 +4996,9 @@
       <c r="I120" s="1" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J120" s="1"/>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
         <v>127</v>
       </c>
@@ -4873,8 +5020,9 @@
         <v>16148</v>
       </c>
       <c r="I121" s="1"/>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J121" s="1"/>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>128</v>
       </c>
@@ -4896,8 +5044,9 @@
         <v>16152</v>
       </c>
       <c r="I122" s="1"/>
-    </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J122" s="1"/>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
         <v>129</v>
       </c>
@@ -4919,8 +5068,9 @@
         <v>16156</v>
       </c>
       <c r="I123" s="1"/>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J123" s="1"/>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
         <v>130</v>
       </c>
@@ -4945,8 +5095,9 @@
         <v>16160</v>
       </c>
       <c r="I124" s="1"/>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J124" s="1"/>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
         <v>131</v>
       </c>
@@ -4974,8 +5125,9 @@
         <v>17172</v>
       </c>
       <c r="I125" s="1"/>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J125" s="1"/>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="4" t="s">
         <v>132</v>
       </c>
@@ -5003,8 +5155,9 @@
         <v>17520</v>
       </c>
       <c r="I126" s="1"/>
-    </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J126" s="1"/>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="4" t="s">
         <v>133</v>
       </c>
@@ -5026,8 +5179,9 @@
         <v>17520</v>
       </c>
       <c r="I127" s="1"/>
-    </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J127" s="1"/>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
         <v>134</v>
       </c>
@@ -5049,8 +5203,9 @@
         <v>17532</v>
       </c>
       <c r="I128" s="1"/>
-    </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J128" s="1"/>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="4" t="s">
         <v>135</v>
       </c>
@@ -5072,8 +5227,9 @@
         <v>17544</v>
       </c>
       <c r="I129" s="1"/>
-    </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J129" s="1"/>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="4" t="s">
         <v>136</v>
       </c>
@@ -5095,8 +5251,9 @@
         <v>17556</v>
       </c>
       <c r="I130" s="1"/>
-    </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J130" s="1"/>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
         <v>137</v>
       </c>
@@ -5118,8 +5275,9 @@
         <v>17568</v>
       </c>
       <c r="I131" s="1"/>
-    </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J131" s="1"/>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="4" t="s">
         <v>138</v>
       </c>
@@ -5141,8 +5299,9 @@
         <v>17580</v>
       </c>
       <c r="I132" s="1"/>
-    </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J132" s="1"/>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="4" t="s">
         <v>139</v>
       </c>
@@ -5164,8 +5323,9 @@
         <v>17592</v>
       </c>
       <c r="I133" s="1"/>
-    </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J133" s="1"/>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="4" t="s">
         <v>140</v>
       </c>
@@ -5187,8 +5347,9 @@
         <v>17604</v>
       </c>
       <c r="I134" s="1"/>
-    </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J134" s="1"/>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
         <v>141</v>
       </c>
@@ -5210,8 +5371,9 @@
         <v>17616</v>
       </c>
       <c r="I135" s="1"/>
-    </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J135" s="1"/>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="4" t="s">
         <v>142</v>
       </c>
@@ -5233,8 +5395,9 @@
         <v>17628</v>
       </c>
       <c r="I136" s="1"/>
-    </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J136" s="1"/>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
         <v>143</v>
       </c>
@@ -5256,8 +5419,9 @@
         <v>17640</v>
       </c>
       <c r="I137" s="1"/>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J137" s="1"/>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
         <v>144</v>
       </c>
@@ -5279,8 +5443,9 @@
         <v>17652</v>
       </c>
       <c r="I138" s="1"/>
-    </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J138" s="1"/>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
         <v>145</v>
       </c>
@@ -5302,8 +5467,9 @@
         <v>17664</v>
       </c>
       <c r="I139" s="1"/>
-    </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J139" s="1"/>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="4" t="s">
         <v>146</v>
       </c>
@@ -5331,8 +5497,9 @@
         <v>17688</v>
       </c>
       <c r="I140" s="1"/>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J140" s="1"/>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="4" t="s">
         <v>147</v>
       </c>
@@ -5354,8 +5521,9 @@
         <v>17688</v>
       </c>
       <c r="I141" s="1"/>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J141" s="1"/>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="4" t="s">
         <v>148</v>
       </c>
@@ -5377,8 +5545,9 @@
         <v>17700</v>
       </c>
       <c r="I142" s="1"/>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J142" s="1"/>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="4" t="s">
         <v>149</v>
       </c>
@@ -5406,8 +5575,9 @@
         <v>18052</v>
       </c>
       <c r="I143" s="1"/>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J143" s="1"/>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="4" t="s">
         <v>150</v>
       </c>
@@ -5435,8 +5605,9 @@
         <v>19220</v>
       </c>
       <c r="I144" s="1"/>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J144" s="1"/>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="4" t="s">
         <v>151</v>
       </c>
@@ -5464,8 +5635,9 @@
         <v>19248</v>
       </c>
       <c r="I145" s="1"/>
-    </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J145" s="1"/>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="4" t="s">
         <v>152</v>
       </c>
@@ -5487,8 +5659,9 @@
         <v>19248</v>
       </c>
       <c r="I146" s="1"/>
-    </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J146" s="1"/>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="4" t="s">
         <v>153</v>
       </c>
@@ -5513,8 +5686,9 @@
         <v>19252</v>
       </c>
       <c r="I147" s="1"/>
-    </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J147" s="1"/>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="4" t="s">
         <v>154</v>
       </c>
@@ -5536,8 +5710,9 @@
         <v>19256</v>
       </c>
       <c r="I148" s="1"/>
-    </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J148" s="1"/>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="4" t="s">
         <v>155</v>
       </c>
@@ -5562,8 +5737,9 @@
         <v>19260</v>
       </c>
       <c r="I149" s="1"/>
-    </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J149" s="1"/>
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150" s="4" t="s">
         <v>156</v>
       </c>
@@ -5585,8 +5761,9 @@
         <v>19264</v>
       </c>
       <c r="I150" s="1"/>
-    </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J150" s="1"/>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="4" t="s">
         <v>157</v>
       </c>
@@ -5608,8 +5785,9 @@
         <v>19272</v>
       </c>
       <c r="I151" s="1"/>
-    </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J151" s="1"/>
+    </row>
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
         <v>158</v>
       </c>
@@ -5631,8 +5809,9 @@
         <v>19276</v>
       </c>
       <c r="I152" s="1"/>
-    </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J152" s="1"/>
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
         <v>159</v>
       </c>
@@ -5654,8 +5833,9 @@
         <v>19280</v>
       </c>
       <c r="I153" s="1"/>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J153" s="1"/>
+    </row>
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
         <v>160</v>
       </c>
@@ -5677,8 +5857,9 @@
         <v>19284</v>
       </c>
       <c r="I154" s="1"/>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J154" s="1"/>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
         <v>161</v>
       </c>
@@ -5700,8 +5881,9 @@
         <v>19288</v>
       </c>
       <c r="I155" s="1"/>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J155" s="1"/>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
         <v>162</v>
       </c>
@@ -5726,8 +5908,9 @@
         <v>19292</v>
       </c>
       <c r="I156" s="1"/>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J156" s="1"/>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
         <v>163</v>
       </c>
@@ -5749,8 +5932,9 @@
         <v>19296</v>
       </c>
       <c r="I157" s="1"/>
-    </row>
-    <row r="158" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J157" s="1"/>
+    </row>
+    <row r="158" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="4" t="s">
         <v>164</v>
       </c>
@@ -5775,8 +5959,9 @@
         <v>19300</v>
       </c>
       <c r="I158" s="1"/>
-    </row>
-    <row r="159" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J158" s="1"/>
+    </row>
+    <row r="159" spans="1:10" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="5" t="s">
         <v>165</v>
       </c>
@@ -5798,10 +5983,13 @@
         <v>19304</v>
       </c>
       <c r="I159" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="160" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+      <c r="J159" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A160" s="4" t="s">
         <v>166</v>
       </c>
@@ -5823,8 +6011,9 @@
         <v>19308</v>
       </c>
       <c r="I160" s="1"/>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J160" s="1"/>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
         <v>167</v>
       </c>
@@ -5846,8 +6035,9 @@
         <v>19312</v>
       </c>
       <c r="I161" s="1"/>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J161" s="1"/>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
         <v>168</v>
       </c>
@@ -5872,8 +6062,9 @@
         <v>19316</v>
       </c>
       <c r="I162" s="1"/>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J162" s="1"/>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
         <v>169</v>
       </c>
@@ -5898,8 +6089,11 @@
         <v>19320</v>
       </c>
       <c r="I163" s="1"/>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J163" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
         <v>170</v>
       </c>
@@ -5924,8 +6118,9 @@
         <v>19324</v>
       </c>
       <c r="I164" s="1"/>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J164" s="1"/>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
         <v>171</v>
       </c>
@@ -5950,8 +6145,9 @@
         <v>19328</v>
       </c>
       <c r="I165" s="1"/>
-    </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J165" s="1"/>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
         <v>172</v>
       </c>
@@ -5973,8 +6169,9 @@
         <v>19332</v>
       </c>
       <c r="I166" s="1"/>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J166" s="1"/>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="4" t="s">
         <v>173</v>
       </c>
@@ -6002,8 +6199,9 @@
         <v>19376</v>
       </c>
       <c r="I167" s="1"/>
-    </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J167" s="1"/>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
         <v>174</v>
       </c>
@@ -6025,8 +6223,9 @@
         <v>19376</v>
       </c>
       <c r="I168" s="1"/>
-    </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J168" s="1"/>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="4" t="s">
         <v>175</v>
       </c>
@@ -6051,8 +6250,9 @@
         <v>19388</v>
       </c>
       <c r="I169" s="1"/>
-    </row>
-    <row r="170" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J169" s="1"/>
+    </row>
+    <row r="170" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A170" s="4" t="s">
         <v>176</v>
       </c>
@@ -6080,10 +6280,11 @@
         <v>19432</v>
       </c>
       <c r="I170" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="171" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+      <c r="J170" s="1"/>
+    </row>
+    <row r="171" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="4" t="s">
         <v>177</v>
       </c>
@@ -6110,8 +6311,9 @@
       <c r="I171" s="1" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="172" spans="1:9" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J171" s="1"/>
+    </row>
+    <row r="172" spans="1:10" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="5" t="s">
         <v>178</v>
       </c>
@@ -6133,10 +6335,13 @@
         <v>19436</v>
       </c>
       <c r="I172" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="173" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+      <c r="J172" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
         <v>179</v>
       </c>
@@ -6158,8 +6363,9 @@
         <v>19440</v>
       </c>
       <c r="I173" s="1"/>
-    </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J173" s="1"/>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174" s="4" t="s">
         <v>180</v>
       </c>
@@ -6181,8 +6387,9 @@
         <v>19444</v>
       </c>
       <c r="I174" s="1"/>
-    </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J174" s="1"/>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175" s="4" t="s">
         <v>181</v>
       </c>
@@ -6204,8 +6411,11 @@
         <v>19448</v>
       </c>
       <c r="I175" s="1"/>
-    </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J175" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
         <v>182</v>
       </c>
@@ -6227,8 +6437,9 @@
         <v>19452</v>
       </c>
       <c r="I176" s="1"/>
-    </row>
-    <row r="177" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J176" s="1"/>
+    </row>
+    <row r="177" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="4" t="s">
         <v>183</v>
       </c>
@@ -6250,8 +6461,9 @@
         <v>19456</v>
       </c>
       <c r="I177" s="1"/>
-    </row>
-    <row r="178" spans="1:9" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J177" s="1"/>
+    </row>
+    <row r="178" spans="1:10" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="5" t="s">
         <v>184</v>
       </c>
@@ -6276,10 +6488,11 @@
         <v>19460</v>
       </c>
       <c r="I178" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="179" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+      <c r="J178" s="1"/>
+    </row>
+    <row r="179" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A179" s="4" t="s">
         <v>185</v>
       </c>
@@ -6301,8 +6514,9 @@
         <v>19464</v>
       </c>
       <c r="I179" s="1"/>
-    </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J179" s="1"/>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A180" s="4" t="s">
         <v>186</v>
       </c>
@@ -6324,8 +6538,11 @@
         <v>19468</v>
       </c>
       <c r="I180" s="1"/>
-    </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J180" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A181" s="4" t="s">
         <v>187</v>
       </c>
@@ -6350,8 +6567,9 @@
         <v>19472</v>
       </c>
       <c r="I181" s="1"/>
-    </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J181" s="1"/>
+    </row>
+    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A182" s="4" t="s">
         <v>188</v>
       </c>
@@ -6373,8 +6591,9 @@
         <v>19476</v>
       </c>
       <c r="I182" s="1"/>
-    </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J182" s="1"/>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
         <v>189</v>
       </c>
@@ -6399,8 +6618,9 @@
         <v>19480</v>
       </c>
       <c r="I183" s="1"/>
-    </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J183" s="1"/>
+    </row>
+    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
         <v>190</v>
       </c>
@@ -6422,8 +6642,9 @@
         <v>19484</v>
       </c>
       <c r="I184" s="1"/>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J184" s="1"/>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A185" s="4" t="s">
         <v>191</v>
       </c>
@@ -6445,8 +6666,9 @@
         <v>19488</v>
       </c>
       <c r="I185" s="1"/>
-    </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J185" s="1"/>
+    </row>
+    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
         <v>192</v>
       </c>
@@ -6468,8 +6690,9 @@
         <v>19492</v>
       </c>
       <c r="I186" s="1"/>
-    </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J186" s="1"/>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A187" s="4" t="s">
         <v>193</v>
       </c>
@@ -6494,8 +6717,9 @@
         <v>19496</v>
       </c>
       <c r="I187" s="1"/>
-    </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J187" s="1"/>
+    </row>
+    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A188" s="4" t="s">
         <v>194</v>
       </c>
@@ -6523,8 +6747,9 @@
         <v>19504</v>
       </c>
       <c r="I188" s="1"/>
-    </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J188" s="1"/>
+    </row>
+    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A189" s="4" t="s">
         <v>195</v>
       </c>
@@ -6546,8 +6771,9 @@
         <v>19504</v>
       </c>
       <c r="I189" s="1"/>
-    </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J189" s="1"/>
+    </row>
+    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A190" s="4" t="s">
         <v>196</v>
       </c>
@@ -6569,8 +6795,9 @@
         <v>19508</v>
       </c>
       <c r="I190" s="1"/>
-    </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J190" s="1"/>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A191" s="4" t="s">
         <v>197</v>
       </c>
@@ -6598,8 +6825,9 @@
         <v>20192</v>
       </c>
       <c r="I191" s="1"/>
-    </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J191" s="1"/>
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A192" s="4" t="s">
         <v>198</v>
       </c>
@@ -6621,8 +6849,9 @@
         <v>20192</v>
       </c>
       <c r="I192" s="1"/>
-    </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J192" s="1"/>
+    </row>
+    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
         <v>199</v>
       </c>
@@ -6644,8 +6873,9 @@
         <v>20272</v>
       </c>
       <c r="I193" s="1"/>
-    </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J193" s="1"/>
+    </row>
+    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A194" s="4" t="s">
         <v>200</v>
       </c>
@@ -6673,8 +6903,9 @@
         <v>20292</v>
       </c>
       <c r="I194" s="1"/>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J194" s="1"/>
+    </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A195" s="4" t="s">
         <v>201</v>
       </c>
@@ -6696,8 +6927,9 @@
         <v>20292</v>
       </c>
       <c r="I195" s="1"/>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J195" s="1"/>
+    </row>
+    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A196" s="4" t="s">
         <v>202</v>
       </c>
@@ -6725,8 +6957,9 @@
         <v>20460</v>
       </c>
       <c r="I196" s="1"/>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J196" s="1"/>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A197" s="4" t="s">
         <v>203</v>
       </c>
@@ -6748,8 +6981,9 @@
         <v>20460</v>
       </c>
       <c r="I197" s="1"/>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J197" s="1"/>
+    </row>
+    <row r="198" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
         <v>204</v>
       </c>
@@ -6774,8 +7008,9 @@
         <v>20464</v>
       </c>
       <c r="I198" s="1"/>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J198" s="1"/>
+    </row>
+    <row r="199" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A199" s="4" t="s">
         <v>205</v>
       </c>
@@ -6797,8 +7032,9 @@
         <v>20468</v>
       </c>
       <c r="I199" s="1"/>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J199" s="1"/>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A200" s="4" t="s">
         <v>206</v>
       </c>
@@ -6823,8 +7059,9 @@
         <v>20472</v>
       </c>
       <c r="I200" s="1"/>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J200" s="1"/>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A201" s="4" t="s">
         <v>207</v>
       </c>
@@ -6846,8 +7083,9 @@
         <v>20476</v>
       </c>
       <c r="I201" s="1"/>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J201" s="1"/>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A202" s="4" t="s">
         <v>208</v>
       </c>
@@ -6875,8 +7113,9 @@
         <v>20500</v>
       </c>
       <c r="I202" s="1"/>
-    </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J202" s="1"/>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
         <v>209</v>
       </c>
@@ -6898,8 +7137,9 @@
         <v>20500</v>
       </c>
       <c r="I203" s="1"/>
-    </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J203" s="1"/>
+    </row>
+    <row r="204" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A204" s="4" t="s">
         <v>210</v>
       </c>
@@ -6921,8 +7161,9 @@
         <v>20504</v>
       </c>
       <c r="I204" s="1"/>
-    </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J204" s="1"/>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A205" s="4" t="s">
         <v>211</v>
       </c>
@@ -6950,8 +7191,9 @@
         <v>20604</v>
       </c>
       <c r="I205" s="1"/>
-    </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J205" s="1"/>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A206" s="4" t="s">
         <v>212</v>
       </c>
@@ -6973,8 +7215,9 @@
         <v>20604</v>
       </c>
       <c r="I206" s="1"/>
-    </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J206" s="1"/>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A207" s="4" t="s">
         <v>213</v>
       </c>
@@ -7002,8 +7245,9 @@
         <v>20644</v>
       </c>
       <c r="I207" s="1"/>
-    </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J207" s="1"/>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A208" s="4" t="s">
         <v>214</v>
       </c>
@@ -7025,8 +7269,9 @@
         <v>20644</v>
       </c>
       <c r="I208" s="1"/>
-    </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J208" s="1"/>
+    </row>
+    <row r="209" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A209" s="4" t="s">
         <v>215</v>
       </c>
@@ -7051,8 +7296,9 @@
         <v>20648</v>
       </c>
       <c r="I209" s="1"/>
-    </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J209" s="1"/>
+    </row>
+    <row r="210" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A210" s="4" t="s">
         <v>216</v>
       </c>
@@ -7077,8 +7323,9 @@
         <v>20652</v>
       </c>
       <c r="I210" s="1"/>
-    </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J210" s="1"/>
+    </row>
+    <row r="211" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A211" s="4" t="s">
         <v>217</v>
       </c>
@@ -7100,8 +7347,9 @@
         <v>20656</v>
       </c>
       <c r="I211" s="1"/>
-    </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J211" s="1"/>
+    </row>
+    <row r="212" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A212" s="4" t="s">
         <v>218</v>
       </c>
@@ -7126,8 +7374,9 @@
         <v>20660</v>
       </c>
       <c r="I212" s="1"/>
-    </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J212" s="1"/>
+    </row>
+    <row r="213" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A213" s="4" t="s">
         <v>219</v>
       </c>
@@ -7149,8 +7398,9 @@
         <v>20664</v>
       </c>
       <c r="I213" s="1"/>
-    </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J213" s="1"/>
+    </row>
+    <row r="214" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A214" s="4" t="s">
         <v>220</v>
       </c>
@@ -7172,8 +7422,9 @@
         <v>20668</v>
       </c>
       <c r="I214" s="1"/>
-    </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J214" s="1"/>
+    </row>
+    <row r="215" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A215" s="4" t="s">
         <v>221</v>
       </c>
@@ -7198,8 +7449,9 @@
         <v>20672</v>
       </c>
       <c r="I215" s="1"/>
-    </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J215" s="1"/>
+    </row>
+    <row r="216" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A216" s="4" t="s">
         <v>222</v>
       </c>
@@ -7221,8 +7473,9 @@
         <v>20676</v>
       </c>
       <c r="I216" s="1"/>
-    </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J216" s="1"/>
+    </row>
+    <row r="217" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A217" s="4" t="s">
         <v>223</v>
       </c>
@@ -7244,8 +7497,9 @@
         <v>20680</v>
       </c>
       <c r="I217" s="1"/>
-    </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J217" s="1"/>
+    </row>
+    <row r="218" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A218" s="4" t="s">
         <v>224</v>
       </c>
@@ -7270,8 +7524,9 @@
         <v>20684</v>
       </c>
       <c r="I218" s="1"/>
-    </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J218" s="1"/>
+    </row>
+    <row r="219" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A219" s="4" t="s">
         <v>225</v>
       </c>
@@ -7293,8 +7548,9 @@
         <v>20688</v>
       </c>
       <c r="I219" s="1"/>
-    </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J219" s="1"/>
+    </row>
+    <row r="220" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A220" s="4" t="s">
         <v>226</v>
       </c>
@@ -7316,8 +7572,9 @@
         <v>20692</v>
       </c>
       <c r="I220" s="1"/>
-    </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J220" s="1"/>
+    </row>
+    <row r="221" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A221" s="4" t="s">
         <v>227</v>
       </c>
@@ -7342,8 +7599,9 @@
         <v>20712</v>
       </c>
       <c r="I221" s="1"/>
-    </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J221" s="1"/>
+    </row>
+    <row r="222" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A222" s="4" t="s">
         <v>228</v>
       </c>
@@ -7365,8 +7623,9 @@
         <v>20716</v>
       </c>
       <c r="I222" s="1"/>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J222" s="1"/>
+    </row>
+    <row r="223" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A223" s="4" t="s">
         <v>229</v>
       </c>
@@ -7391,8 +7650,9 @@
         <v>20720</v>
       </c>
       <c r="I223" s="1"/>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J223" s="1"/>
+    </row>
+    <row r="224" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A224" s="4" t="s">
         <v>230</v>
       </c>
@@ -7414,8 +7674,9 @@
         <v>20724</v>
       </c>
       <c r="I224" s="1"/>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J224" s="1"/>
+    </row>
+    <row r="225" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A225" s="4" t="s">
         <v>231</v>
       </c>
@@ -7437,8 +7698,9 @@
         <v>20728</v>
       </c>
       <c r="I225" s="1"/>
-    </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J225" s="1"/>
+    </row>
+    <row r="226" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A226" s="4" t="s">
         <v>232</v>
       </c>
@@ -7460,8 +7722,9 @@
         <v>20732</v>
       </c>
       <c r="I226" s="1"/>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J226" s="1"/>
+    </row>
+    <row r="227" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A227" s="4" t="s">
         <v>233</v>
       </c>
@@ -7483,8 +7746,9 @@
         <v>20736</v>
       </c>
       <c r="I227" s="1"/>
-    </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J227" s="1"/>
+    </row>
+    <row r="228" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
         <v>234</v>
       </c>
@@ -7506,8 +7770,9 @@
         <v>20740</v>
       </c>
       <c r="I228" s="1"/>
-    </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J228" s="1"/>
+    </row>
+    <row r="229" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A229" s="4" t="s">
         <v>235</v>
       </c>
@@ -7529,8 +7794,9 @@
         <v>20744</v>
       </c>
       <c r="I229" s="1"/>
-    </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J229" s="1"/>
+    </row>
+    <row r="230" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A230" s="4" t="s">
         <v>236</v>
       </c>
@@ -7555,8 +7821,9 @@
         <v>20748</v>
       </c>
       <c r="I230" s="1"/>
-    </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J230" s="1"/>
+    </row>
+    <row r="231" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A231" s="4" t="s">
         <v>237</v>
       </c>
@@ -7578,8 +7845,9 @@
         <v>20752</v>
       </c>
       <c r="I231" s="1"/>
-    </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J231" s="1"/>
+    </row>
+    <row r="232" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
         <v>238</v>
       </c>
@@ -7601,8 +7869,9 @@
         <v>20756</v>
       </c>
       <c r="I232" s="1"/>
-    </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J232" s="1"/>
+    </row>
+    <row r="233" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
         <v>239</v>
       </c>
@@ -7624,8 +7893,9 @@
         <v>20760</v>
       </c>
       <c r="I233" s="1"/>
-    </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J233" s="1"/>
+    </row>
+    <row r="234" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A234" s="4" t="s">
         <v>240</v>
       </c>
@@ -7653,8 +7923,9 @@
         <v>20820</v>
       </c>
       <c r="I234" s="1"/>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J234" s="1"/>
+    </row>
+    <row r="235" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A235" s="4" t="s">
         <v>241</v>
       </c>
@@ -7676,8 +7947,9 @@
         <v>20820</v>
       </c>
       <c r="I235" s="1"/>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J235" s="1"/>
+    </row>
+    <row r="236" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A236" s="4" t="s">
         <v>242</v>
       </c>
@@ -7699,8 +7971,9 @@
         <v>20824</v>
       </c>
       <c r="I236" s="1"/>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J236" s="1"/>
+    </row>
+    <row r="237" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A237" s="4" t="s">
         <v>243</v>
       </c>
@@ -7728,8 +8001,9 @@
         <v>21568</v>
       </c>
       <c r="I237" s="1"/>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J237" s="1"/>
+    </row>
+    <row r="238" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
         <v>244</v>
       </c>
@@ -7754,8 +8028,9 @@
         <v>21568</v>
       </c>
       <c r="I238" s="1"/>
-    </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J238" s="1"/>
+    </row>
+    <row r="239" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A239" s="4" t="s">
         <v>245</v>
       </c>
@@ -7777,8 +8052,9 @@
         <v>21572</v>
       </c>
       <c r="I239" s="1"/>
-    </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J239" s="1"/>
+    </row>
+    <row r="240" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A240" s="4" t="s">
         <v>246</v>
       </c>
@@ -7805,8 +8081,9 @@
       <c r="I240" s="1" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J240" s="1"/>
+    </row>
+    <row r="241" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A241" s="4" t="s">
         <v>247</v>
       </c>
@@ -7828,8 +8105,9 @@
         <v>21640</v>
       </c>
       <c r="I241" s="1"/>
-    </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J241" s="1"/>
+    </row>
+    <row r="242" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A242" s="4" t="s">
         <v>248</v>
       </c>
@@ -7851,8 +8129,9 @@
         <v>21664</v>
       </c>
       <c r="I242" s="1"/>
-    </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J242" s="1"/>
+    </row>
+    <row r="243" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A243" s="4" t="s">
         <v>249</v>
       </c>
@@ -7877,8 +8156,9 @@
         <v>21680</v>
       </c>
       <c r="I243" s="1"/>
-    </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J243" s="1"/>
+    </row>
+    <row r="244" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A244" s="4" t="s">
         <v>250</v>
       </c>
@@ -7900,8 +8180,9 @@
         <v>21684</v>
       </c>
       <c r="I244" s="1"/>
-    </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J244" s="1"/>
+    </row>
+    <row r="245" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A245" s="4" t="s">
         <v>251</v>
       </c>
@@ -7923,8 +8204,9 @@
         <v>21748</v>
       </c>
       <c r="I245" s="1"/>
-    </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J245" s="1"/>
+    </row>
+    <row r="246" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A246" s="4" t="s">
         <v>252</v>
       </c>
@@ -7946,8 +8228,9 @@
         <v>21772</v>
       </c>
       <c r="I246" s="1"/>
-    </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J246" s="1"/>
+    </row>
+    <row r="247" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A247" s="4" t="s">
         <v>253</v>
       </c>
@@ -7975,8 +8258,9 @@
         <v>21812</v>
       </c>
       <c r="I247" s="1"/>
-    </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J247" s="1"/>
+    </row>
+    <row r="248" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
         <v>254</v>
       </c>
@@ -8001,8 +8285,9 @@
         <v>21812</v>
       </c>
       <c r="I248" s="1"/>
-    </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J248" s="1"/>
+    </row>
+    <row r="249" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A249" s="4" t="s">
         <v>255</v>
       </c>
@@ -8026,8 +8311,9 @@
       <c r="I249" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J249" s="1"/>
+    </row>
+    <row r="250" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A250" s="4" t="s">
         <v>256</v>
       </c>
@@ -8051,8 +8337,9 @@
       <c r="I250" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J250" s="1"/>
+    </row>
+    <row r="251" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A251" s="4" t="s">
         <v>257</v>
       </c>
@@ -8074,12 +8361,13 @@
         <v>21944</v>
       </c>
       <c r="I251" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="252" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+      <c r="J251" s="1"/>
+    </row>
+    <row r="252" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A252" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B252" t="s">
         <v>18</v>
@@ -8099,12 +8387,13 @@
         <v>22008</v>
       </c>
       <c r="I252" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="253" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+        <v>282</v>
+      </c>
+      <c r="J252" s="1"/>
+    </row>
+    <row r="253" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A253" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B253" t="s">
         <v>18</v>
@@ -8124,10 +8413,11 @@
         <v>22072</v>
       </c>
       <c r="I253" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+      <c r="J253" s="1"/>
+    </row>
+    <row r="254" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A254" s="4" t="s">
         <v>258</v>
       </c>
@@ -8151,8 +8441,9 @@
       <c r="I254" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J254" s="1"/>
+    </row>
+    <row r="255" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A255" s="4" t="s">
         <v>259</v>
       </c>
@@ -8176,8 +8467,9 @@
       <c r="I255" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J255" s="1"/>
+    </row>
+    <row r="256" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A256" s="4" t="s">
         <v>260</v>
       </c>
@@ -8201,8 +8493,9 @@
       <c r="I256" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J256" s="1"/>
+    </row>
+    <row r="257" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A257" s="4" t="s">
         <v>261</v>
       </c>
@@ -8226,8 +8519,9 @@
       <c r="I257" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J257" s="1"/>
+    </row>
+    <row r="258" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A258" s="4" t="s">
         <v>262</v>
       </c>
@@ -8255,8 +8549,9 @@
         <v>22476</v>
       </c>
       <c r="I258" s="1"/>
-    </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J258" s="1"/>
+    </row>
+    <row r="259" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A259" s="4" t="s">
         <v>263</v>
       </c>
@@ -8281,8 +8576,9 @@
         <v>22476</v>
       </c>
       <c r="I259" s="1"/>
-    </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J259" s="1"/>
+    </row>
+    <row r="260" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A260" s="4" t="s">
         <v>264</v>
       </c>
@@ -8307,8 +8603,9 @@
         <v>22480</v>
       </c>
       <c r="I260" s="1"/>
-    </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J260" s="1"/>
+    </row>
+    <row r="261" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A261" s="4" t="s">
         <v>265</v>
       </c>
@@ -8336,8 +8633,9 @@
         <v>22556</v>
       </c>
       <c r="I261" s="1"/>
-    </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J261" s="1"/>
+    </row>
+    <row r="262" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A262" s="4" t="s">
         <v>266</v>
       </c>
@@ -8362,8 +8660,9 @@
         <v>22556</v>
       </c>
       <c r="I262" s="1"/>
-    </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J262" s="1"/>
+    </row>
+    <row r="263" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A263" s="4" t="s">
         <v>267</v>
       </c>
@@ -8388,8 +8687,9 @@
         <v>22560</v>
       </c>
       <c r="I263" s="1"/>
-    </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J263" s="1"/>
+    </row>
+    <row r="264" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A264" s="4" t="s">
         <v>268</v>
       </c>
@@ -8417,8 +8717,9 @@
         <v>22572</v>
       </c>
       <c r="I264" s="1"/>
-    </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J264" s="1"/>
+    </row>
+    <row r="265" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A265" s="4" t="s">
         <v>269</v>
       </c>
@@ -8443,8 +8744,9 @@
         <v>22572</v>
       </c>
       <c r="I265" s="1"/>
-    </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J265" s="1"/>
+    </row>
+    <row r="266" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A266" s="4" t="s">
         <v>270</v>
       </c>
@@ -8472,8 +8774,9 @@
         <v>22588</v>
       </c>
       <c r="I266" s="1"/>
-    </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J266" s="1"/>
+    </row>
+    <row r="267" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A267" s="4" t="s">
         <v>271</v>
       </c>
@@ -8498,8 +8801,9 @@
         <v>22588</v>
       </c>
       <c r="I267" s="1"/>
-    </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J267" s="1"/>
+    </row>
+    <row r="268" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
         <v>272</v>
       </c>
@@ -8527,8 +8831,9 @@
         <v>22624</v>
       </c>
       <c r="I268" s="1"/>
-    </row>
-    <row r="269" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J268" s="1"/>
+    </row>
+    <row r="269" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E269" s="2">
         <f>SUM(E2:E268)</f>
         <v>22624</v>
@@ -8542,7 +8847,17 @@
         <v>22624</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="270" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="271" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B271" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="272" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B272" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B1:E269" xr:uid="{C3C11D8C-D518-42C3-A7D3-6BD4B138053A}"/>
   <conditionalFormatting sqref="G2:G268">

</xml_diff>

<commit_message>
Rename GTR2MemOps -> Gtr2ProgMemOps to prepare for Gtr2SharMemOps
</commit_message>
<xml_diff>
--- a/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
+++ b/etc/Gtr2MemGridVehicleSlot-memory-mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\matt\Code\gtr2-memory-operations-tool-wpf\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FBD10A-08EF-4557-826C-F7D4B68CA63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA655752-8E38-4BE8-882C-A13A6DE79A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17532" yWindow="3972" windowWidth="26064" windowHeight="15900" xr2:uid="{A748CD8A-F26B-4A5C-81FA-994BF5EB8B3B}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="296">
   <si>
     <t>Name</t>
   </si>
@@ -981,6 +981,9 @@
   </si>
   <si>
     <t>Note: Field Length = 40 not 36 (confirmed reading driver names correctly in Gtr2MemOpsTool gui app)</t>
+  </si>
+  <si>
+    <t>Value is its own memory address if valid or 0xFFFFFFFF to indicate the linked list is terminated.</t>
   </si>
 </sst>
 </file>
@@ -1925,7 +1928,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1945,7 +1948,9 @@
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="I2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>295</v>
+      </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>